<commit_message>
Grade categories: point-based, total exactly 1000 (asserted in generator)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1682,7 +1682,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E3">
         <f>(B3-C3)*D3</f>
@@ -1702,7 +1702,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="E4">
         <f>(B4-C4)*D4</f>
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E5">
         <f>(B5-C5)*D5</f>

</xml_diff>

<commit_message>
Calendar rework: in-class quiz days, flex day, Michael's grade scheme
- Quizzes are dedicated in-class Friday days (Sep 25, Oct 23, Nov 20),
  matching the previous prof, instead of annotations on lecture days
- Flex day Fri Oct 9 (week 5, where her snow day fell); absorbs snow /
  Mountain Day
- Removed invented tail days (FFT/review padding); her 39 spring slots
  now map 1:1 onto the 39 fall meetings, calendar exactly full
- Grade categories synced from Michael's 2026-08-11 xlsx edits into the
  generator (35/300/25/450/190 = 1000; Non-Newtonian Scientist = one HW
  via =D3); recorded in README and syllabus TODO

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>Finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
+          <t>Eigenvalues and eigenvectors, continued</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -689,12 +689,12 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>The two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -737,10 +737,14 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Practice / review day</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>Setting up 1D and 2D integrals</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>5.1-5.2</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
@@ -789,12 +793,12 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; the gradient</t>
+          <t>Cartesian 2D integrals; polar coordinates</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.4</t>
+          <t>5.3-5.4</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -837,12 +841,12 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Work, path integrals, and the gradient theorem</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
@@ -872,66 +876,58 @@
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 13</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>Gradient, divergence, curl</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>8.5-8.7</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Practice / review day</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>WHW10</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 3 (Ch 6, 5)</t>
-        </is>
-      </c>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Fri Sep 25</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Jupyter notebook exercise: ODEs in Python</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>WHW03</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="n">
         <v>11</v>
       </c>
@@ -945,12 +941,12 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Divergence, curl, and the Laplacian</t>
+          <t>Vector and scalar fields; the gradient</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>8.6-8.7</t>
+          <t>8.1-8.4</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
@@ -970,12 +966,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Heaviside, Dirac delta, and the Laplace transform</t>
+          <t>Jupyter notebook exercise: ODEs in Python</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>10.10</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
@@ -993,12 +989,12 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Work, path integrals, and the gradient theorem</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
@@ -1018,76 +1014,72 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Using Laplace transforms to solve ODEs</t>
+          <t>Heaviside, Dirac delta, and the Laplace transform</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>10.11</t>
+          <t>10.10</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Conservative vector fields</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>8.11</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Fri Oct 2</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Complex numbers: basic properties</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>3.1-3.4</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Using Laplace transforms to solve ODEs</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>10.11</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>WHW04</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 1 (Ch 1 + 10)</t>
-        </is>
-      </c>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="n">
         <v>12</v>
       </c>
@@ -1101,12 +1093,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Gradient, divergence, curl</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>8.5-8.7</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1126,12 +1118,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Euler's formula; complex ODEs</t>
+          <t>Complex numbers: basic properties</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.1-3.4</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1166,12 +1158,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Linear approximations</t>
+          <t>Euler's formula; complex ODEs</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2.1-2.2</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1206,14 +1198,10 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Maclaurin series</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
+          <t>Flex day (snow / Mountain Day buffer)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>WHW05</t>
@@ -1233,12 +1221,12 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains</t>
+          <t>Divergence, curl, and the Laplacian</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>8.6-8.7</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
@@ -1273,12 +1261,12 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Fourier series with complex exponentials</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>8.9-8.10</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1298,12 +1286,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Taylor series; finding one series from another</t>
+          <t>Linear approximations</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5</t>
+          <t>2.1-2.2</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1321,12 +1309,12 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1350,12 +1338,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Properties of matrices</t>
+          <t>Maclaurin series</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1377,12 +1365,12 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>PDEs continued; separation of variables preview</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -1402,12 +1390,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Matrix x column; vector transformations</t>
+          <t>Taylor series; finding one series from another</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>6.3-6.4</t>
+          <t>2.4-2.5</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1425,10 +1413,14 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Python: FFTs and real data</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
+          <t>Fourier series: different periods, finite domains</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
     </row>
@@ -1446,12 +1438,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
+          <t>Properties of matrices</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>6.5-6.7</t>
+          <t>6.1-6.2</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1469,10 +1461,14 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Review / flex day</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr"/>
+          <t>Fourier series with complex exponentials</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
           <t>WHW13</t>
@@ -1494,14 +1490,10 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Finding eigenvalues and eigenvectors</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
+          <t>Quiz 2 (Ch 10, 3, 2)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
           <t>WHW07</t>
@@ -1525,10 +1517,14 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Review and wrap-up</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr"/>
+          <t>Intro to PDEs: the heat equation</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>11.1-11.2</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr"/>
     </row>
@@ -1546,12 +1542,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
+          <t>Matrix x column; vector transformations</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.3-6.4</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1590,12 +1586,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>The two-coupled-oscillator problem</t>
+          <t>Matrix multiplication; identity, determinant, inverse</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>6.5-6.7</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1612,7 +1608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1659,7 +1655,7 @@
         <v>39</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1682,7 +1678,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E3">
         <f>(B3-C3)*D3</f>
@@ -1692,17 +1688,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quizzes</t>
+          <t>Non-Newtonian Scientist</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="n">
-        <v>110</v>
+      <c r="D4">
+        <f>D3</f>
+        <v/>
       </c>
       <c r="E4">
         <f>(B4-C4)*D4</f>
@@ -1712,17 +1709,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Final exam</t>
+          <t>Quizzes</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E5">
         <f>(B5-C5)*D5</f>
@@ -1732,11 +1729,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Final exam</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>190</v>
+      </c>
+      <c r="E6">
+        <f>(B6-C6)*D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E6">
-        <f>SUM(E2:E5)</f>
+      <c r="E7">
+        <f>SUM(E2:E6)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
F2026 calendar: fix polar-coordinates reading label (5.6, not 5.3-5.4)
Verified against the Felder & Felder table of contents: 5.3-5.4 are
Cartesian double integrals; polar is 5.6. The wrong label was inherited
verbatim from the S26 schedule grid. Regenerated the xlsx.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Grade Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4</t>
+          <t>5.3-5.4, 5.6</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
F2026 calendar: encode all 2026-08-17 decisions
- Review day -> cylindrical/spherical coordinate-systems day (5.5, 5.7)
- Feynman Vol II Ch 2-3 assigned BEFORE Felder 8.6-8.7 (geometric
  definitions of div/curl first); Ch 3 also cited on the theorems day
- Fourier series compressed to 2 days (9.1-9.3, 9.4-9.5)
- PDEs protected with 2 days (11.1-11.2+11.4, then 11.3)
- Fourier transforms (9.6) ride the Dec 14 finale, taught graphically
- 2.6-2.7 convergence cut with Appendix C pointer on the Taylor day
- Non-Newtonian Scientist due mid-semester, Mon Oct 26 (EXTRA_DUE)
- README + TODO updated (decisions locked; PCCIs Gary's way; next big
  task = re-cut WHWs to the new calendar + per-day PCCI assignments)

Regenerated PHY210 F2026 Calendar.xlsx; 39-slot and 1000-point asserts
pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -889,10 +889,14 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Practice / review day</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>5.5, 5.7; App. D</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>WHW10</t>
@@ -1093,12 +1097,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Gradient, divergence, curl</t>
+          <t>Divergence and curl, geometrically</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>8.5-8.7</t>
+          <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1266,7 +1270,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10</t>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1395,7 +1399,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5</t>
+          <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1413,12 +1417,12 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains</t>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.4-9.5</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
@@ -1461,12 +1465,12 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Fourier series with complex exponentials</t>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>11.1-11.2, 11.4</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1517,12 +1521,12 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation</t>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2</t>
+          <t>11.3, 9.6</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
@@ -1550,7 +1554,11 @@
           <t>6.3-6.4</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>

</xml_diff>

<commit_message>
F2026 calendar: PCCI column + WHW Problem Lists tab
PCCIs (Gary-Felder style, decided 2026-08-17): 35 assignments, one per
non-quiz/non-flex class day, inline on the Schedule tab -- mostly the
day's Discovery Exercise, every number attested in a predecessor's
actual assignment (Gary's PCCI schedules, Gillian's WHW forms, Casey's
in-class sets). New 'WHW Problem Lists' tab: 13 weekly tiered lists
(Warm-up/Essentials/Depth) re-cut from Gillian's transcribed S26 forms
onto the F2026 week boundaries, with attested supplements for the
units S26 lacked (coordinates day, Feynman/8.x days, Ch 10 split);
Gillian's standing preamble at the top for Moodle copy-paste. Asserts:
PCCIs only on class days, never quiz days; WHW tab numbers match the
calendar's 13 Friday WHWs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -89,6 +90,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -457,23 +461,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,45 +510,55 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Topics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Reading Due</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
@@ -570,35 +586,45 @@
           <t>1.1-1.2</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="n">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Fri Oct 30</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Finding eigenvalues and eigenvectors</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>WHW08</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -624,33 +650,43 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>DE 1.2.1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>WHW01</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="n">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="K3" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 2</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Eigenvalues and eigenvectors, continued</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>6.166</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -674,31 +710,41 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.3.1 Part 1</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 4</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>The two-coupled-oscillator problem</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>6.9</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -722,35 +768,45 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.5.1 Parts 1-5</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="n">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="K5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 6</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>5.1-5.2</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -776,33 +832,43 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>DE 1.6.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>WHW02</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="n">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 9</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Cartesian 2D integrals; polar coordinates</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>5.3-5.4, 5.6</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -826,31 +892,41 @@
           <t>1.6</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1.166</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="n">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 11</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Line integrals and surface integrals</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>5.8, 5.10</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -874,35 +950,45 @@
           <t>10.2</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10.1, 10.3</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="n">
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 13</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>5.5, 5.7; App. D</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>WHW10</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -922,39 +1008,45 @@
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>WHW03</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Quiz 1 (Ch 1)</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 16</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Vector and scalar fields; the gradient</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>8.1-8.4</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.2.1 Parts 5-6</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -978,31 +1070,41 @@
           <t>10.2</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="n">
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 18</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Work, path integrals, and the gradient theorem</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1026,31 +1128,37 @@
           <t>10.10</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10.5, 10.8</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="I11" s="3" t="n">
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="J11" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="K11" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr"/>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
@@ -1080,33 +1188,43 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>10.216</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>WHW04</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="n">
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Divergence and curl, geometrically</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1130,23 +1248,29 @@
           <t>3.1-3.4</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.2.1</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="I13" s="4" t="n"/>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1170,23 +1294,29 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.4.1</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="I14" s="4" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Fri Nov 27</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1206,35 +1336,41 @@
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>WHW05</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="n">
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 30</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Divergence, curl, and the Laplacian</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>8.6-8.7</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.6.1 Parts 1-9</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1252,29 +1388,35 @@
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="I16" s="2" t="n">
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 2</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1298,35 +1440,45 @@
           <t>2.1-2.2</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="n">
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 4</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Conservative vector fields</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>8.11</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>WHW12</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1352,33 +1504,43 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>WHW06</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="n">
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 7</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Introduction to Fourier series</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>9.1-9.3</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.2.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1402,31 +1564,41 @@
           <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2.209</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="n">
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="K19" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 9</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>9.4-9.5</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1450,35 +1622,45 @@
           <t>6.1-6.2</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="n">
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="K20" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 11</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>11.1-11.2, 11.4</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>WHW13</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1498,39 +1680,45 @@
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>WHW07</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="J21" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="K21" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>11.3, 9.6</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1556,25 +1744,31 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>Non-Newtonian Scientist due</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="I22" s="4" t="n"/>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 8, 9, 11 + redemptions)</t>
         </is>
@@ -1602,8 +1796,13 @@
           <t>6.5-6.7</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1611,6 +1810,486 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>The following problems are useful practice for the week. I recommend starting with the warm-ups. If they're too easy, move on to Essentials. If you're interested in the Depth content, you can add those problems as well. You are not expected to do all the problems. DE x.y.1 = the Discovery Exercise of section x.y. Answers to odd problems: felderbooks.com/mathmethods (Appendix M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>WHW</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Covers</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Warm-up</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Essentials</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Depth</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WHW01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 11</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Intro to ODEs (1.1-1.2)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.17, 1.19</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.18, 1.20, 1.21, 1.25</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.33, 1.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>WHW02</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 18</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants (1.3); separation of variables (1.5)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.39, 1.41, 1.43. Separation of variables: 1.90, 1.91, 1.93, 1.95</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.38, 1.46, 1.58. Separation of variables: 1.103</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.60. Separation of variables: 1.105</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>WHW03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 25</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check, superposition (1.6); linear operators (10.2)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.108, 1.109. Sec 10.2: 10.1, 10.3, 10.5, 10.8</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.111, 1.113, 1.117, 1.122, 1.29. Sec 10.2: 10.13, 10.26, 10.31</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.125, 1.131. Sec 10.2: 10.32, 10.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>WHW04</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 2</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ODEs in Python; Heaviside, Dirac, Laplace (10.10)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>10.216, 10.217, 10.218</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.10: 10.219, 10.223, 10.230, 10.242</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on posit.smith.edu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>WHW05</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 9</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Solving ODEs with Laplace transforms (10.11); complex numbers and Euler (3.1-3.5)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.246, 10.248. Complex numbers: 3.17, 3.19, 3.47. Euler / complex ODE: 3.59, 3.65, 3.92</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.252, 10.261, 10.263, 10.264. Complex numbers: 3.49, 3.54. Euler / complex ODE: 3.77, 3.94, 3.95</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.270, 10.272, 10.274. Complex numbers: 3.45, 3.56. Euler / complex ODE: 3.85, 3.107</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 16</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations (2.1-2.2); Maclaurin series (2.3)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations: 2.6, 2.7, 2.16</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series: 2.31, 2.35, 2.37</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series: 2.86, 2.87</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>WHW07</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 23</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series (2.4-2.5); matrices and the three-spring problem (6.1-6.2)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series: 2.41. The three-spring problem: 6.2. Normal modes: 6.3. Matrices: 6.19</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin/Taylor: 2.47, 2.49, 2.53, 2.55, 2.57, 2.67. The three-spring problem: 6.7, 6.17. Normal modes: 6.9. Matrices: 6.21, 6.23</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series: 2.71, 2.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column, basis, matrix times matrix, identity, inverse, determinants (6.3-6.7)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column: 6.27, 6.29, 6.31. Matrix-matrix: 6.69. Identity and inverse: DE 6.6.1, 6.97. Determinants: 6.127, 6.129</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column: 6.35, 6.41. Matrix-matrix: 6.81, 6.89, 6.91. Identity and inverse: 6.99, 6.101, 6.103, 6.107, 6.109, 6.119, 6.121, 6.123. Determinants: 6.133, 6.139</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Basis and transformations: 6.45, 6.53, 6.55, 6.57, 6.61. Determinants: 6.147, 6.161</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 6</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvalues and eigenvectors (6.8); coupled oscillators (6.9)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.166, 6.170, 6.172, 6.175</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.171, 6.173, 6.177</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.179, 6.181, 6.185</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 13</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up integrals; Cartesian doubles, polar; line and surface integrals (5.1-5.4, 5.6, 5.8, 5.10)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D integrals: 5.1-5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D integrals: 5.7, 5.9, 5.11, 5.19, 5.23. Single integrals in multiple dimensions: 5.35, 5.43, 5.45, 5.51. Cartesian rectangular: 5.71, 5.75, 5.77. Cartesian non-rectangular: 5.83, 5.85, 5.97, 5.101. Line integrals: 5.199, 5.201, 5.215, 5.217, 5.229. Surface integrals: 5.256, 5.257, 5.263</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Line integrals: 5.223, 5.225, 5.235</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>WHW11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Cylindrical and spherical coordinates (5.5, 5.7); fields, potential, gradient (8.1-8.5)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: DE 8.2.1, 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Spherical coordinates: 5.181, 5.187. Polar and cylindrical: 5.129, 5.137, 5.147, 5.153. Scalar and vector fields: 8.5, 8.7, 8.9, 8.17, 8.19, 8.21, 8.25. Potential in 1D: 8.37, 8.41, 8.43. From potential to gradients: 8.57, 8.59, 8.65</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Polar and cylindrical: 5.157, 5.169, 5.171, 5.193. All coordinates: 5.165</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 4</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl, Feynman and Felder (Feynman II 2-3, 8.6-8.7); divergence theorem and Stokes' theorem (8.9-8.10)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl by inspection: 8.84, 8.86. Divergence theorem: DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl: 8.88, 8.90, 8.94, 8.98, 8.102, 8.110. Divergence theorem: 8.147, 8.151, 8.155, 8.157. Stokes' theorem: 8.159, 8.163, 8.165, 8.169, 8.171</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>8.106. Write out Feynman's flux-through-a-tiny-cube derivation of the divergence theorem in your own words, with pictures</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields (8.11); Fourier series (9.1-9.5)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: DE 8.11.1. Fourier series: DE 9.2.1, 9.5, 9.7, 9.9</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: 8.178. Fourier series: 9.15, 9.17, 9.23, 9.27, 9.29, 9.33</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: 8.173, 8.177, 8.179, 8.181. Different periods and finite domains: 9.38, 9.41, 9.47. Complex Fourier series: 9.60, 9.62, 9.66</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1627,27 +2306,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Drop</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Points Each</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Total Points</t>
         </is>

</xml_diff>

<commit_message>
F2026 calendar: dedupe WHW lists against PCCI assignments
Problems promoted to graded PCCIs are no longer repeated in the WHW
practice tiers (10.1/10.3/10.5/10.8, 10.216, 6.2, 6.166, 6.175, 5.1,
DE 8.2.1, DE 8.9.1, DE 8.11.1, DE 9.2.1); convention noted in the
generator comments. Regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1947,7 +1947,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Guess and check: 1.108, 1.109. Sec 10.2: 10.1, 10.3, 10.5, 10.8</t>
+          <t>Guess and check: 1.108, 1.109</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>10.216, 10.217, 10.218</t>
+          <t>10.217, 10.218</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Taylor series: 2.41. The three-spring problem: 6.2. Normal modes: 6.3. Matrices: 6.19</t>
+          <t>Taylor series: 2.41. Normal modes: 6.3. Matrices: 6.19</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Eigenvectors &amp; eigenvalues: 6.166, 6.170, 6.172, 6.175</t>
+          <t>Eigenvectors &amp; eigenvalues: 6.170, 6.172</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D integrals: 5.1-5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
+          <t>Setting up 1D integrals: 5.2, 5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: DE 8.2.1, 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
+          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Divergence and curl by inspection: 8.84, 8.86. Divergence theorem: DE 8.9.1</t>
+          <t>Divergence and curl by inspection: 8.84, 8.86</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Conservative fields: DE 8.11.1. Fourier series: DE 9.2.1, 9.5, 9.7, 9.9</t>
+          <t>Fourier series: 9.5, 9.7, 9.9</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
F2026 calendar: no PCCI on day 1; first PCCI (syllabus+advice) day 2
Nobody has the syllabus before the first class. Matches Gary's actual
pattern (first PCCI on day 2). DE 1.2.1 dropped rather than shifted:
class 01 does its content live. DE 1.3.1 unchanged on Mon Sep 14,
still priming the arbitrary-constants day. 34 PCCIs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -586,11 +586,7 @@
           <t>1.1-1.2</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
@@ -650,7 +646,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>DE 1.2.1</t>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Grading rebalance: participation 2 pts/day (70), quizzes 140, final 185
Michael's 2026-08-25 decision, made in the syllabus: more credit for
attendance/participation. Generator constants updated (asserts still
require exactly 1000), xlsx regenerated, MoodleBuildSpec gradebook
and TODO item 8 synced.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -2341,7 +2341,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <f>(B2-C2)*D2</f>
@@ -2402,7 +2402,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E5">
         <f>(B5-C5)*D5</f>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E6">
         <f>(B6-C6)*D6</f>

</xml_diff>

<commit_message>
Calendar: single-block 'Schedule (web)' tab for the Moodle embed
The two-block Schedule sheet is ~1600px wide; the embed needs one
continuous ~800px table.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule (web)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1811,6 +1812,1350 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reading Due</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>HW Due</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Exams</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 9</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Syllabus; SHO and overview of differential equations</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1.1-1.2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 11</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Generating ODEs from physical situations</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1.1-1.2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>WHW01</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 14</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants; initial conditions</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 16</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Separation of variables</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.5.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 18</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.6.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>WHW02</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 21</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Linearity, homogeneity, superposition</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1.166</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 23</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Methods of solving ODEs: guess and check</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10.1, 10.3</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Fri Sep 25</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>WHW03</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Jupyter notebook exercise: ODEs in Python</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 30</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Heaviside, Dirac delta, and the Laplace transform</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>10.10</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10.5, 10.8</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 2</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Using Laplace transforms to solve ODEs</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>10.11</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>10.216</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>WHW04</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 5</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Complex numbers: basic properties</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>3.1-3.4</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.2.1</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Euler's formula; complex ODEs</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.4.1</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 9</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Flex day (snow / Mountain Day buffer)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>WHW05</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Mon Oct 12</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>No class - Autumn recess</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 14</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2.1-2.2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 16</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 19</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series; finding one series from another</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2.4-2.5 (convergence: App. C)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2.209</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Properties of matrices</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>6.1-6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fri Oct 23</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 2 (Ch 10, 3, 2)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>WHW07</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 2 (Ch 10, 3, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 26</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Matrix x column; vector transformations</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>6.3-6.4</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 28</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Matrix multiplication; identity, determinant, inverse</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>6.5-6.7</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 30</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Finding eigenvalues and eigenvectors</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 2</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvalues and eigenvectors, continued</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>6.166</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 4</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The two-coupled-oscillator problem</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 6</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D and 2D integrals</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>5.1-5.2</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 9</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Cartesian 2D integrals; polar coordinates</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>5.3-5.4, 5.6</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 11</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Line integrals and surface integrals</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>5.8, 5.10</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 13</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>5.5, 5.7; App. D</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 16</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Vector and scalar fields; the gradient</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>8.1-8.4</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.2.1 Parts 5-6</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 18</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Work, path integrals, and the gradient theorem</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>WHW11</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 23</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl, geometrically</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Feynman Vol II Ch 2-3</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Wed Nov 25</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 27</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 30</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Divergence, curl, and the Laplacian</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>8.6-8.7</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.6.1 Parts 1-9</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Wed Dec 2</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Divergence theorem; Stokes' theorem</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 4</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Conservative vector fields</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>8.11</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Mon Dec 7</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Introduction to Fourier series</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>9.1-9.3</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.2.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Wed Dec 9</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>9.4-9.5</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>11.1-11.2, 11.4</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Mon Dec 14</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>11.3, 9.6</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Sat Dec 19</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Final exam period Dec 19-22 (registrar schedules)</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Final (Ch 8, 9, 11 + redemptions)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2285,7 +3630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Calendar: chunked Schedule (web) tab for the half-semester embed
Two chunks split at fall break, each with its own header row; the
generator prints the embed ranges every run. Spec gains the full
embed/switch/re-import procedure.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1812,7 +1812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2310,97 +2310,109 @@
       <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 14</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Linear approximations</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2.1-2.2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.2.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Reading Due</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>HW Due</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>Exams</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Fri Oct 16</t>
+          <t>Wed Oct 14</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Maclaurin series</t>
+          <t>Linear approximations</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.1-2.2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>DE 2.3.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>WHW06</t>
-        </is>
-      </c>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Mon Oct 19</t>
+          <t>Fri Oct 16</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Taylor series; finding one series from another</t>
+          <t>Maclaurin series</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2.209</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -2408,123 +2420,123 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 21</t>
+          <t>Mon Oct 19</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Properties of matrices</t>
+          <t>Taylor series; finding one series from another</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>2.209</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Properties of matrices</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>6.1-6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Fri Oct 23</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>WHW07</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 26</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Matrix x column; vector transformations</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>6.3-6.4</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.3.1</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Non-Newtonian Scientist due</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
+          <t>Matrix x column; vector transformations</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.5-6.7</t>
+          <t>6.3-6.4</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>DE 6.5.1</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2532,50 +2544,46 @@
         <v>8</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Fri Oct 30</t>
+          <t>Wed Oct 28</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Finding eigenvalues and eigenvectors</t>
+          <t>Matrix multiplication; identity, determinant, inverse</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.5-6.7</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>DE 6.8.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>WHW08</t>
-        </is>
-      </c>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 2</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
+          <t>Finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2585,10 +2593,14 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>6.166</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -2596,26 +2608,26 @@
         <v>9</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 4</t>
+          <t>Mon Nov 2</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>The two-coupled-oscillator problem</t>
+          <t>Eigenvalues and eigenvectors, continued</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>6.175</t>
+          <t>6.166</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -2626,63 +2638,63 @@
         <v>9</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Fri Nov 6</t>
+          <t>Wed Nov 4</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>The two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>WHW09</t>
-        </is>
-      </c>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 9</t>
+          <t>Fri Nov 6</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4, 5.6</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>DE 5.4.1</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2690,26 +2702,26 @@
         <v>10</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 11</t>
+          <t>Mon Nov 9</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Cartesian 2D integrals; polar coordinates</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>5.3-5.4, 5.6</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>5.163 parts a and d</t>
+          <t>DE 5.4.1</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -2720,63 +2732,63 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Fri Nov 13</t>
+          <t>Wed Nov 11</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>WHW10</t>
-        </is>
-      </c>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 16</t>
+          <t>Fri Nov 13</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; the gradient</t>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.4</t>
+          <t>5.5, 5.7; App. D</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DE 8.2.1 Parts 5-6</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2784,115 +2796,127 @@
         <v>11</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 18</t>
+          <t>Mon Nov 16</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Work, path integrals, and the gradient theorem</t>
+          <t>Vector and scalar fields; the gradient</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1-8.4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>DE 8.4.1</t>
+          <t>DE 8.2.1 Parts 5-6</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 18</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Work, path integrals, and the gradient theorem</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
+    <row r="35">
+      <c r="A35" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Divergence and curl, geometrically</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Wed Nov 25</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
       <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Fri Nov 27</t>
+          <t>Wed Nov 25</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2906,60 +2930,48 @@
       <c r="H36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 30</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Divergence, curl, and the Laplacian</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>8.6-8.7</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.6.1 Parts 1-9</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 27</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wed Dec 2</t>
+          <t>Mon Nov 30</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Divergence, curl, and the Laplacian</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10; Feynman Vol II Ch 3</t>
+          <t>8.6-8.7</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DE 8.9.1</t>
+          <t>DE 8.6.1 Parts 1-9</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -2970,63 +2982,63 @@
         <v>13</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Fri Dec 4</t>
+          <t>Wed Dec 2</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Conservative vector fields</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>WHW12</t>
-        </is>
-      </c>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mon Dec 7</t>
+          <t>Fri Dec 4</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DE 9.2.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
       <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
@@ -3034,26 +3046,26 @@
         <v>14</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Wed Dec 9</t>
+          <t>Mon Dec 7</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains, complex exponentials</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>9.4-9.5</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>DE 9.4.1 Part 1</t>
+          <t>DE 9.2.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
@@ -3064,82 +3076,112 @@
         <v>14</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Fri Dec 11</t>
+          <t>Wed Dec 9</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2, 11.4</t>
+          <t>9.4-9.5</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>DE 11.2.1 Parts 1-2</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>WHW13</t>
-        </is>
-      </c>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>11.1-11.2, 11.4</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>11.3, 9.6</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>DE 11.3.1 Part 1</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 8, 9, 11 + redemptions)</t>
         </is>

</xml_diff>

<commit_message>
Calendar: one canonical Schedule tab (chunked single block)
Drop the two-side-by-side-blocks print layout -- it existed to serve
the embed-half-at-a-time practice, which the chunked ranges now do.
Header cells wrap; Week/Class/Reading Due columns widened.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule (web)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -81,9 +80,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -96,6 +97,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -462,1364 +464,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Topics</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Reading Due</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>PCCI</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>HW Due</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Exams</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Topics</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Reading Due</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>PCCI</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>HW Due</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Exams</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 9</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Syllabus; SHO and overview of differential equations</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1.1-1.2</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 30</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Finding eigenvalues and eigenvectors</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.8.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>WHW08</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Fri Sep 11</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Generating ODEs from physical situations</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>1.1-1.2</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>WHW01</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 2</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>6.166</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 14</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Arbitrary constants; initial conditions</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.3.1 Part 1</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 4</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>The two-coupled-oscillator problem</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>6.9</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>6.175</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 16</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Separation of variables</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.5.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Fri Nov 6</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Setting up 1D and 2D integrals</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>5.1-5.2</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>WHW09</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Fri Sep 18</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Guess and check</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.6.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>WHW02</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 9</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>5.3-5.4, 5.6</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>DE 5.4.1</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 21</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Linearity, homogeneity, superposition</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1.166</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 11</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Line integrals and surface integrals</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>5.8, 5.10</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>5.163 parts a and d</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 23</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Methods of solving ODEs: guess and check</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>10.1, 10.3</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Fri Nov 13</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>5.5, 5.7; App. D</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>DE 5.7.1 Parts 1-4</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>WHW10</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Fri Sep 25</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 1 (Ch 1)</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>WHW03</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 1 (Ch 1)</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 16</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Vector and scalar fields; the gradient</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>8.1-8.4</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.2.1 Parts 5-6</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 28</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Jupyter notebook exercise: ODEs in Python</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 18</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Work, path integrals, and the gradient theorem</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.4.1</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 30</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Heaviside, Dirac delta, and the Laplace transform</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>10.10</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>10.5, 10.8</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="J11" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Fri Nov 20</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 3 (Ch 6, 5)</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr"/>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t>WHW11</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 3 (Ch 6, 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 2</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Using Laplace transforms to solve ODEs</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>10.11</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>10.216</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>WHW04</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 23</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Divergence and curl, geometrically</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>Feynman Vol II Ch 2-3</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 5</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Complex numbers: basic properties</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>3.1-3.4</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>DE 3.2.1</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Wed Nov 25</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 7</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Euler's formula; complex ODEs</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>DE 3.4.1</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Fri Nov 27</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 9</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Flex day (snow / Mountain Day buffer)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>WHW05</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 30</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Divergence, curl, and the Laplacian</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>8.6-8.7</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.6.1 Parts 1-9</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Mon Oct 12</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>No class - Autumn recess</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Wed Dec 2</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Divergence theorem; Stokes' theorem</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>8.9-8.10; Feynman Vol II Ch 3</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.9.1</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 14</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Linear approximations</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2.1-2.2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.2.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K17" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Fri Dec 4</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Conservative vector fields</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>8.11</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>WHW12</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 16</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Maclaurin series</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.3.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>WHW06</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Mon Dec 7</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>Introduction to Fourier series</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>9.1-9.3</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.2.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 19</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Taylor series; finding one series from another</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>2.209</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K19" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Wed Dec 9</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Fourier series: different periods, finite domains, complex exponentials</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>9.4-9.5</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.4.1 Part 1</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 21</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Properties of matrices</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>6.1-6.2</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K20" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Fri Dec 11</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>11.1-11.2, 11.4</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.2.1 Parts 1-2</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>WHW13</t>
-        </is>
-      </c>
-      <c r="Q20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Fri Oct 23</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 2 (Ch 10, 3, 2)</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>WHW07</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 2 (Ch 10, 3, 2)</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K21" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>Mon Dec 14</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Normal modes of the wave equation; Fourier transforms</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>11.3, 9.6</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.3.1 Part 1</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 26</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Matrix x column; vector transformations</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>6.3-6.4</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.3.1</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Non-Newtonian Scientist due</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Sat Dec 19</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>Final exam period Dec 19-22 (registrar schedules)</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
-      <c r="Q22" s="4" t="inlineStr">
-        <is>
-          <t>Final (Ch 8, 9, 11 + redemptions)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 28</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>6.5-6.7</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.5.1</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -3192,7 +1844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3217,32 +1869,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>WHW</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Covers</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Warm-up</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Depth</t>
         </is>
@@ -3672,7 +2324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3689,27 +2341,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Drop</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Points Each</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Total Points</t>
         </is>

</xml_diff>

<commit_message>
Platform: jupyterhub.smith.edu replaces posit (syllabus, generator, spec, notes)
Same switch as PHY 317 (2026-09-07): posit's Workbench cannot start
sessions and has no packages; the hub has the full stack and ipywidgets.
Syllabus (two places), the Sep 28 PCCI and WHW04 depth item in the
generator, MoodleBuildSpec (with the hub lessons: VPN off campus, pin
%matplotlib inline because the hub defaults to ipympl), TODO item 27
resolved, ComputationalProblems.md's scipy caveat lifted (scipy 1.14 is
there), Notebooks2026 README.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+          <t>Log into jupyterhub.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Redo the class notebook's exercises from scratch in a fresh notebook on posit.smith.edu</t>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WHW01: 1.36 (by computer) moved to WHW04; guard against by-computer problems before the Python class
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>ODEs: 1.33, 1.36</t>
+          <t>ODEs: 1.33</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu</t>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu. Sec 1.2: 1.36 (compound interest, by computer; moved here from WHW01)</t>
         </is>
       </c>
     </row>

</xml_diff>